<commit_message>
Alteração no arquivo FLM-FTE-BOM-01
</commit_message>
<xml_diff>
--- a/PCB/BOM/FLM-FTE-BOM-01.xlsx
+++ b/PCB/BOM/FLM-FTE-BOM-01.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luish\Desktop\Projetos Faculdade\Fonte_Linear_12V\PCB\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26C5FB20-2427-4238-99F0-1CDE6487F159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="60" windowWidth="27795" windowHeight="12345"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCB-ER-FTE-12V1A" sheetId="1" r:id="rId1"/>
@@ -14,17 +20,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="98">
   <si>
     <t>Footprint</t>
   </si>
   <si>
-    <t>4700uF/25V</t>
-  </si>
-  <si>
-    <t>Capacitor_THT:CP_Radial_D16.0mm_P7.50mm</t>
-  </si>
-  <si>
     <t>0,1uF/50V</t>
   </si>
   <si>
@@ -139,9 +139,6 @@
     <t>Resistor_THT:R_Axial_DIN0207_L6.3mm_D2.5mm_P7.62mm_Horizontal</t>
   </si>
   <si>
-    <t>R2,R6</t>
-  </si>
-  <si>
     <t>10K 1/4W</t>
   </si>
   <si>
@@ -190,9 +187,6 @@
     <t>U1</t>
   </si>
   <si>
-    <t>ESP32-WROOM-32E</t>
-  </si>
-  <si>
     <t>PCB-GERAL:ESP32-WROOM-32E-N8</t>
   </si>
   <si>
@@ -209,6 +203,114 @@
   </si>
   <si>
     <t>Valor</t>
+  </si>
+  <si>
+    <t>0,22R/5W</t>
+  </si>
+  <si>
+    <t>Resistor_THT:R_Axial_DIN0516_L15.5mm_D5.0mm_P5.08mm_Vertical</t>
+  </si>
+  <si>
+    <t>REG1</t>
+  </si>
+  <si>
+    <t>LM7812</t>
+  </si>
+  <si>
+    <t>BPSC-4</t>
+  </si>
+  <si>
+    <t>C2,C4,C9,C10,C11,C13</t>
+  </si>
+  <si>
+    <t>MCS-6</t>
+  </si>
+  <si>
+    <t>REG3</t>
+  </si>
+  <si>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>10uF/16V</t>
+  </si>
+  <si>
+    <t>C1,C5</t>
+  </si>
+  <si>
+    <t>4700uF/35V</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>R4,R6,R7</t>
+  </si>
+  <si>
+    <t>RF1,RF2</t>
+  </si>
+  <si>
+    <t>RG1</t>
+  </si>
+  <si>
+    <t>U2</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>R12</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>C3,C8</t>
+  </si>
+  <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>R8,R9,R13</t>
+  </si>
+  <si>
+    <t>0,33R/5W</t>
+  </si>
+  <si>
+    <t>15K</t>
+  </si>
+  <si>
+    <t>11K</t>
+  </si>
+  <si>
+    <t>LM358N</t>
+  </si>
+  <si>
+    <t>14K 1/4W</t>
+  </si>
+  <si>
+    <t>BPSC-2</t>
+  </si>
+  <si>
+    <t>ESP32-WROOM-32E-N8</t>
+  </si>
+  <si>
+    <t>100uF/50V</t>
+  </si>
+  <si>
+    <t>Resistor_THT:R_Axial_DIN0207_L6.3mm_D2.5mm_P2.54mm_Vertical</t>
+  </si>
+  <si>
+    <t>PCB-CI:DIP8</t>
+  </si>
+  <si>
+    <t>PCB-CI:LM78XX</t>
+  </si>
+  <si>
+    <t>Connector_PinSocket_2.54mm:PinSocket_1x02_P2.54mm_Vertical</t>
+  </si>
+  <si>
+    <t>Capacitor_THT:CP_Radial_D18.0mm_P7.50mm</t>
   </si>
   <si>
     <r>
@@ -232,130 +334,43 @@
       </rPr>
       <t xml:space="preserve"> Fonte Linear Regulada 12V</t>
     </r>
-  </si>
-  <si>
-    <t>Cód. Sisgem:</t>
-  </si>
-  <si>
-    <t>0,22R/5W</t>
-  </si>
-  <si>
-    <t>Resistor_THT:R_Axial_DIN0516_L15.5mm_D5.0mm_P5.08mm_Vertical</t>
-  </si>
-  <si>
-    <t>010136</t>
-  </si>
-  <si>
-    <t>R5,R12</t>
-  </si>
-  <si>
-    <t>010183</t>
-  </si>
-  <si>
-    <t>010286</t>
-  </si>
-  <si>
-    <t>REG1</t>
-  </si>
-  <si>
-    <t>LM7812</t>
-  </si>
-  <si>
-    <t>PCB-CI:TO-220</t>
-  </si>
-  <si>
-    <t>112805</t>
-  </si>
-  <si>
-    <t>BPSC-4</t>
-  </si>
-  <si>
-    <t>113331</t>
-  </si>
-  <si>
-    <t>C2,C4,C9,C10,C11,C13</t>
-  </si>
-  <si>
-    <t>114334</t>
-  </si>
-  <si>
-    <t>114642</t>
-  </si>
-  <si>
-    <t>114715</t>
-  </si>
-  <si>
-    <t>114841</t>
-  </si>
-  <si>
-    <t>MCS-6</t>
-  </si>
-  <si>
-    <t>119911</t>
-  </si>
-  <si>
-    <t>121835</t>
-  </si>
-  <si>
-    <t>REG3</t>
-  </si>
-  <si>
-    <t>130379</t>
-  </si>
-  <si>
-    <t>130411</t>
-  </si>
-  <si>
-    <t>130483</t>
-  </si>
-  <si>
-    <t>L1</t>
-  </si>
-  <si>
-    <t>137742</t>
-  </si>
-  <si>
-    <t>139388</t>
-  </si>
-  <si>
-    <t>C3,C7,C8</t>
-  </si>
-  <si>
-    <t>010121.133</t>
-  </si>
-  <si>
-    <t>10uF/16V</t>
-  </si>
-  <si>
-    <t>010121.290</t>
-  </si>
-  <si>
-    <t>010121.338</t>
-  </si>
-  <si>
-    <t>C1,C5</t>
-  </si>
-  <si>
-    <t>010132.208</t>
-  </si>
-  <si>
-    <t>010132.216</t>
-  </si>
-  <si>
-    <t>010132.240</t>
-  </si>
-  <si>
-    <t>010136.576</t>
-  </si>
-  <si>
-    <t>R3,R8,R9,R13</t>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">Equipe: </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>FLM System</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="20" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -501,6 +516,12 @@
     </font>
     <font>
       <u/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="16"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -848,19 +869,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -896,10 +911,10 @@
     <cellStyle name="Ênfase5" xfId="34" builtinId="45" customBuiltin="1"/>
     <cellStyle name="Ênfase6" xfId="38" builtinId="49" customBuiltin="1"/>
     <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Incorreto" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Neutra" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="Neutro" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Nota" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Ruim" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Saída" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="Texto de Aviso" xfId="14" builtinId="11" customBuiltin="1"/>
     <cellStyle name="Texto Explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
@@ -910,10 +925,7 @@
     <cellStyle name="Título 4" xfId="5" builtinId="19" customBuiltin="1"/>
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="7">
-    <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -921,10 +933,10 @@
       <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -938,28 +950,30 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabela1" displayName="Tabela1" ref="A2:E29" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
-  <autoFilter ref="A2:E29"/>
-  <tableColumns count="5">
-    <tableColumn id="1" name="Cód. Sisgem:" dataDxfId="4"/>
-    <tableColumn id="2" name="Referencia" dataDxfId="3"/>
-    <tableColumn id="3" name="Valor" dataDxfId="2"/>
-    <tableColumn id="4" name="Quantidade" dataDxfId="1"/>
-    <tableColumn id="5" name="Footprint" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabela1" displayName="Tabela1" ref="A2:D36" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A2:D36" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="4">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Referencia" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Valor" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Quantidade" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Footprint" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema do Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Escritório">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -997,7 +1011,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Escritório">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1069,7 +1083,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Escritório">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1242,497 +1256,517 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.28515625" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.5703125" customWidth="1"/>
-    <col min="5" max="5" width="65.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.5703125" customWidth="1"/>
+    <col min="4" max="4" width="65.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="2">
+        <v>3</v>
+      </c>
+      <c r="D6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C9" s="2">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>77</v>
+      </c>
+      <c r="B10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>79</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="2">
+        <v>3</v>
+      </c>
+      <c r="D13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>63</v>
+      </c>
+      <c r="B14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C14" s="2">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="C15" s="2">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>80</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>66</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1" t="s">
+      <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C17" s="2">
+        <v>6</v>
+      </c>
+      <c r="D17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="2">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="2">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>27</v>
+      </c>
+      <c r="B20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C20" s="2">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="2">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="2">
+      <c r="B22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="2">
+        <v>4</v>
+      </c>
+      <c r="D22" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>68</v>
+      </c>
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="2">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C25" s="2">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>69</v>
+      </c>
+      <c r="B26" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="2">
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>54</v>
+      </c>
+      <c r="B27" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" s="2">
+        <v>1</v>
+      </c>
+      <c r="D27" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>81</v>
+      </c>
+      <c r="B28" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" s="2">
         <v>2</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="2">
-        <v>1</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="1" t="s">
+      <c r="D28" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>82</v>
+      </c>
+      <c r="B29" t="s">
+        <v>91</v>
+      </c>
+      <c r="C29" s="2">
+        <v>1</v>
+      </c>
+      <c r="D29" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>8</v>
+      </c>
+      <c r="B30" t="s">
+        <v>70</v>
+      </c>
+      <c r="C30" s="2">
+        <v>1</v>
+      </c>
+      <c r="D30" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="2">
+        <v>1</v>
+      </c>
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B32" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" s="2">
+        <v>2</v>
+      </c>
+      <c r="D32" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" t="s">
+        <v>44</v>
+      </c>
+      <c r="C33" s="2">
+        <v>1</v>
+      </c>
+      <c r="D33" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="B34" t="s">
+        <v>42</v>
+      </c>
+      <c r="C34" s="2">
+        <v>1</v>
+      </c>
+      <c r="D34" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>36</v>
+      </c>
+      <c r="B35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C35" s="2">
+        <v>1</v>
+      </c>
+      <c r="D35" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>83</v>
+      </c>
+      <c r="B36" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="2">
         <v>3</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
-      <c r="B6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D6" s="2">
-        <v>1</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" s="2">
-        <v>2</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="2">
-        <v>3</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D9" s="2">
-        <v>1</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D10" s="2">
-        <v>1</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="2">
-        <v>6</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="2">
-        <v>1</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="D13" s="2">
-        <v>1</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" s="2">
-        <v>1</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D15" s="2">
-        <v>1</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D16" s="2">
-        <v>4</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D17" s="2">
-        <v>1</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D18" s="2">
-        <v>1</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D19" s="2">
-        <v>1</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="2">
-        <v>1</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D21" s="2">
-        <v>1</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="2">
-        <v>3</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D23" s="2">
-        <v>1</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="2">
-        <v>1</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D25" s="2">
-        <v>2</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D26" s="2">
-        <v>1</v>
-      </c>
-      <c r="E26" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D27" s="2">
-        <v>1</v>
-      </c>
-      <c r="E27" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B28" s="1" t="s">
+      <c r="D36" t="s">
         <v>38</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D28" s="2">
-        <v>1</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D29" s="2">
-        <v>4</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>